<commit_message>
Update QA reports with critical API and data persistence findings
Added 18 new test cases from deep functional audit:
- 7 API endpoints return empty/mock data (chat, jobs, workers, listings, bookings, QR verify, payments)
- 8 data persistence failures (avatar, groups, posts, friends, wallet, chat, search not connected to DB)
- 3 security issues (QR verify always true, admin org code unvalidated, in-memory rate limiting)

Updated results: 81 test cases, 58.0% pass rate (47 pass, 34 fail)

https://claude.ai/code/session_01RGfJPwNgYTYKFEZvETDMzN
</commit_message>
<xml_diff>
--- a/QA_Reports/QA_Report.xlsx
+++ b/QA_Reports/QA_Report.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J64"/>
+  <dimension ref="A1:J82"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -2460,9 +2460,585 @@
         <v/>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>TC064</v>
+      </c>
+      <c r="B65" t="str">
+        <v>API</v>
+      </c>
+      <c r="C65" t="str">
+        <v>Chat API</v>
+      </c>
+      <c r="D65" t="str">
+        <v>GET /api/chat returns messages</v>
+      </c>
+      <c r="E65" t="str">
+        <v>API returns messages for given roomId from Supabase</v>
+      </c>
+      <c r="F65" t="str">
+        <v>GET endpoint returns hardcoded empty array: const data: any[] = []. No Supabase query.</v>
+      </c>
+      <c r="G65" t="str">
+        <v>Fail</v>
+      </c>
+      <c r="H65" t="str">
+        <v>API_Chat_EmptyData.png</v>
+      </c>
+      <c r="I65" t="str">
+        <v>Chat API returns empty array regardless of roomId - no DB query</v>
+      </c>
+      <c r="J65" t="str">
+        <v>Implement Supabase query to fetch messages by roomId</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>TC065</v>
+      </c>
+      <c r="B66" t="str">
+        <v>API</v>
+      </c>
+      <c r="C66" t="str">
+        <v>Jobs API</v>
+      </c>
+      <c r="D66" t="str">
+        <v>GET /api/jobs returns jobs</v>
+      </c>
+      <c r="E66" t="str">
+        <v>API returns jobs with category/pagination filters from Supabase</v>
+      </c>
+      <c r="F66" t="str">
+        <v>GET endpoint returns hardcoded empty array: const data: any[] = []. No Supabase query.</v>
+      </c>
+      <c r="G66" t="str">
+        <v>Fail</v>
+      </c>
+      <c r="H66" t="str">
+        <v>API_Jobs_EmptyData.png</v>
+      </c>
+      <c r="I66" t="str">
+        <v>Jobs API returns empty data - DB query not implemented</v>
+      </c>
+      <c r="J66" t="str">
+        <v>Implement Supabase query to fetch jobs with filters</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>TC066</v>
+      </c>
+      <c r="B67" t="str">
+        <v>API</v>
+      </c>
+      <c r="C67" t="str">
+        <v>Workers API</v>
+      </c>
+      <c r="D67" t="str">
+        <v>GET /api/workers returns workers</v>
+      </c>
+      <c r="E67" t="str">
+        <v>API returns worker profiles from Supabase</v>
+      </c>
+      <c r="F67" t="str">
+        <v>Contains TODO comments. Both GET and POST return empty arrays. No Supabase query.</v>
+      </c>
+      <c r="G67" t="str">
+        <v>Fail</v>
+      </c>
+      <c r="H67" t="str">
+        <v>API_Workers_NotImplemented.png</v>
+      </c>
+      <c r="I67" t="str">
+        <v>Worker API is a stub with TODO comments</v>
+      </c>
+      <c r="J67" t="str">
+        <v>Implement Supabase query to worker_profiles table</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>TC067</v>
+      </c>
+      <c r="B68" t="str">
+        <v>API</v>
+      </c>
+      <c r="C68" t="str">
+        <v>Listings API</v>
+      </c>
+      <c r="D68" t="str">
+        <v>GET /api/listings returns listings</v>
+      </c>
+      <c r="E68" t="str">
+        <v>API returns marketplace listings from Supabase</v>
+      </c>
+      <c r="F68" t="str">
+        <v>Contains TODO comments. Returns empty data. No Supabase query.</v>
+      </c>
+      <c r="G68" t="str">
+        <v>Fail</v>
+      </c>
+      <c r="H68" t="str">
+        <v>API_Listings_NotImplemented.png</v>
+      </c>
+      <c r="I68" t="str">
+        <v>Listings API is a stub with TODO comments</v>
+      </c>
+      <c r="J68" t="str">
+        <v>Implement Supabase query to listings table</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>TC068</v>
+      </c>
+      <c r="B69" t="str">
+        <v>API</v>
+      </c>
+      <c r="C69" t="str">
+        <v>Bookings API</v>
+      </c>
+      <c r="D69" t="str">
+        <v>GET /api/bookings returns bookings</v>
+      </c>
+      <c r="E69" t="str">
+        <v>API returns bookings from Supabase</v>
+      </c>
+      <c r="F69" t="str">
+        <v>Contains TODO comments. Returns empty data. No Supabase query.</v>
+      </c>
+      <c r="G69" t="str">
+        <v>Fail</v>
+      </c>
+      <c r="H69" t="str">
+        <v>API_Bookings_NotImplemented.png</v>
+      </c>
+      <c r="I69" t="str">
+        <v>Bookings API is a stub with TODO comments</v>
+      </c>
+      <c r="J69" t="str">
+        <v>Implement Supabase query to bookings table</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>TC069</v>
+      </c>
+      <c r="B70" t="str">
+        <v>API</v>
+      </c>
+      <c r="C70" t="str">
+        <v>QR Verify API</v>
+      </c>
+      <c r="D70" t="str">
+        <v>POST /api/qr/verify validates QR codes</v>
+      </c>
+      <c r="E70" t="str">
+        <v>API validates QR code against stored codes in database</v>
+      </c>
+      <c r="F70" t="str">
+        <v>Always returns {verified: true} without any database verification. Contains TODO comment.</v>
+      </c>
+      <c r="G70" t="str">
+        <v>Fail</v>
+      </c>
+      <c r="H70" t="str">
+        <v>API_QRVerify_AlwaysTrue.png</v>
+      </c>
+      <c r="I70" t="str">
+        <v>SECURITY FLAW: QR verification always returns true without checking DB</v>
+      </c>
+      <c r="J70" t="str">
+        <v>Implement real QR code validation against Supabase stored codes</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>TC070</v>
+      </c>
+      <c r="B71" t="str">
+        <v>API</v>
+      </c>
+      <c r="C71" t="str">
+        <v>Payments API</v>
+      </c>
+      <c r="D71" t="str">
+        <v>POST /api/payments processes payment</v>
+      </c>
+      <c r="E71" t="str">
+        <v>Payment processed through Stripe/Adyen gateway</v>
+      </c>
+      <c r="F71" t="str">
+        <v>Returns mock payment with status "pending". Contains TODO: "Integrate Stripe/Adyen". No real payment processing.</v>
+      </c>
+      <c r="G71" t="str">
+        <v>Fail</v>
+      </c>
+      <c r="H71" t="str">
+        <v>API_Payments_MockOnly.png</v>
+      </c>
+      <c r="I71" t="str">
+        <v>No payment gateway integration - returns mock data</v>
+      </c>
+      <c r="J71" t="str">
+        <v>Integrate Stripe or Adyen PCI-compliant payment provider</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>TC071</v>
+      </c>
+      <c r="B72" t="str">
+        <v>Profile</v>
+      </c>
+      <c r="C72" t="str">
+        <v>Profile Edit</v>
+      </c>
+      <c r="D72" t="str">
+        <v>Avatar upload persists across sessions</v>
+      </c>
+      <c r="E72" t="str">
+        <v>Avatar saved to Supabase storage bucket</v>
+      </c>
+      <c r="F72" t="str">
+        <v>Avatar upload uses FileReader to store as DataURL in localStorage only. Not connected to Supabase storage.</v>
+      </c>
+      <c r="G72" t="str">
+        <v>Fail</v>
+      </c>
+      <c r="H72" t="str">
+        <v>Profile_AvatarNotPersisted.png</v>
+      </c>
+      <c r="I72" t="str">
+        <v>Avatar stored in localStorage, not Supabase storage. Lost on browser clear.</v>
+      </c>
+      <c r="J72" t="str">
+        <v>Connect to uploadAvatar in supabase.ts for persistent storage</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>TC072</v>
+      </c>
+      <c r="B73" t="str">
+        <v>Community</v>
+      </c>
+      <c r="C73" t="str">
+        <v>Community</v>
+      </c>
+      <c r="D73" t="str">
+        <v>Created group persists in database</v>
+      </c>
+      <c r="E73" t="str">
+        <v>New group saved to communities table in Supabase</v>
+      </c>
+      <c r="F73" t="str">
+        <v>handleCreate only validates with AI safety scan and shows success message. Does NOT call createCommunity from supabase.ts.</v>
+      </c>
+      <c r="G73" t="str">
+        <v>Fail</v>
+      </c>
+      <c r="H73" t="str">
+        <v>Community_GroupNotSaved.png</v>
+      </c>
+      <c r="I73" t="str">
+        <v>Group creation UI does not call database save function</v>
+      </c>
+      <c r="J73" t="str">
+        <v>Call createCommunity after successful safety scan</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>TC073</v>
+      </c>
+      <c r="B74" t="str">
+        <v>Community</v>
+      </c>
+      <c r="C74" t="str">
+        <v>Community</v>
+      </c>
+      <c r="D74" t="str">
+        <v>Group post persists in database</v>
+      </c>
+      <c r="E74" t="str">
+        <v>Post saved to posts table with community context</v>
+      </c>
+      <c r="F74" t="str">
+        <v>handlePost scans content but only updates local state. Does NOT call createPost.</v>
+      </c>
+      <c r="G74" t="str">
+        <v>Fail</v>
+      </c>
+      <c r="H74" t="str">
+        <v>Community_PostNotSaved.png</v>
+      </c>
+      <c r="I74" t="str">
+        <v>Community post not saved to database</v>
+      </c>
+      <c r="J74" t="str">
+        <v>Call createPost with community_id after content moderation passes</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>TC074</v>
+      </c>
+      <c r="B75" t="str">
+        <v>Friends</v>
+      </c>
+      <c r="C75" t="str">
+        <v>Friends</v>
+      </c>
+      <c r="D75" t="str">
+        <v>Friend requests persist</v>
+      </c>
+      <c r="E75" t="str">
+        <v>Friend request saved to friend_requests table</v>
+      </c>
+      <c r="F75" t="str">
+        <v>All friend request operations (send/accept/decline) only modify local component state. No Supabase calls.</v>
+      </c>
+      <c r="G75" t="str">
+        <v>Fail</v>
+      </c>
+      <c r="H75" t="str">
+        <v>Friends_RequestsNotPersisted.png</v>
+      </c>
+      <c r="I75" t="str">
+        <v>Friend operations not connected to backend</v>
+      </c>
+      <c r="J75" t="str">
+        <v>Call sendFriendRequest/respondFriendRequest from supabase.ts</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>TC075</v>
+      </c>
+      <c r="B76" t="str">
+        <v>Friends</v>
+      </c>
+      <c r="C76" t="str">
+        <v>Friends</v>
+      </c>
+      <c r="D76" t="str">
+        <v>Blocked users enforced server-side</v>
+      </c>
+      <c r="E76" t="str">
+        <v>Blocked users stored in friend_requests table with blocked status</v>
+      </c>
+      <c r="F76" t="str">
+        <v>Block/unblock only uses localStorage via getBlockedUsers/toggleBlock. Not server-enforced.</v>
+      </c>
+      <c r="G76" t="str">
+        <v>Fail</v>
+      </c>
+      <c r="H76" t="str">
+        <v>Friends_BlockingClientOnly.png</v>
+      </c>
+      <c r="I76" t="str">
+        <v>Blocking is client-side only, can be bypassed via API</v>
+      </c>
+      <c r="J76" t="str">
+        <v>Use respondFriendRequest with blocked status and enforce via RLS</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>TC076</v>
+      </c>
+      <c r="B77" t="str">
+        <v>Wallet</v>
+      </c>
+      <c r="C77" t="str">
+        <v>Wallet</v>
+      </c>
+      <c r="D77" t="str">
+        <v>Wallet shows real balance</v>
+      </c>
+      <c r="E77" t="str">
+        <v>Balance fetched from wallets table in Supabase</v>
+      </c>
+      <c r="F77" t="str">
+        <v>All balance and transaction data is hardcoded in useState. No Supabase calls.</v>
+      </c>
+      <c r="G77" t="str">
+        <v>Fail</v>
+      </c>
+      <c r="H77" t="str">
+        <v>Wallet_DummyData.png</v>
+      </c>
+      <c r="I77" t="str">
+        <v>Wallet uses hardcoded mock data, not connected to database</v>
+      </c>
+      <c r="J77" t="str">
+        <v>Call getWalletBalance and getTransactions from supabase.ts</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>TC077</v>
+      </c>
+      <c r="B78" t="str">
+        <v>Chat</v>
+      </c>
+      <c r="C78" t="str">
+        <v>Chat</v>
+      </c>
+      <c r="D78" t="str">
+        <v>Messages persist across sessions</v>
+      </c>
+      <c r="E78" t="str">
+        <v>Messages saved to messages table via sendMessage</v>
+      </c>
+      <c r="F78" t="str">
+        <v>Messages stored in component state only. No API calls to save. Auto-replies are hardcoded.</v>
+      </c>
+      <c r="G78" t="str">
+        <v>Fail</v>
+      </c>
+      <c r="H78" t="str">
+        <v>Chat_MessagesNotPersisted.png</v>
+      </c>
+      <c r="I78" t="str">
+        <v>Chat messages are ephemeral - lost on page refresh</v>
+      </c>
+      <c r="J78" t="str">
+        <v>Call sendMessage from supabase.ts and subscribe to realtime updates</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>TC078</v>
+      </c>
+      <c r="B79" t="str">
+        <v>Search</v>
+      </c>
+      <c r="C79" t="str">
+        <v>Search</v>
+      </c>
+      <c r="D79" t="str">
+        <v>Search queries real database content</v>
+      </c>
+      <c r="E79" t="str">
+        <v>Search indexes content from Supabase tables</v>
+      </c>
+      <c r="F79" t="str">
+        <v>Search index built from hardcoded DEMO_WORKERS and DEMO_JOBS arrays only. No real DB content.</v>
+      </c>
+      <c r="G79" t="str">
+        <v>Fail</v>
+      </c>
+      <c r="H79" t="str">
+        <v>Search_DemoDataOnly.png</v>
+      </c>
+      <c r="I79" t="str">
+        <v>Search only returns demo/mock data, not real database content</v>
+      </c>
+      <c r="J79" t="str">
+        <v>Build search index from actual Supabase queries</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>TC079</v>
+      </c>
+      <c r="B80" t="str">
+        <v>Search</v>
+      </c>
+      <c r="C80" t="str">
+        <v>Search</v>
+      </c>
+      <c r="D80" t="str">
+        <v>Voice search captures real speech</v>
+      </c>
+      <c r="E80" t="str">
+        <v>Web Speech API captures and converts voice to search query</v>
+      </c>
+      <c r="F80" t="str">
+        <v>Voice button shows "Listening..." for 2 seconds then hardcodes query to "plumber". No real speech recognition.</v>
+      </c>
+      <c r="G80" t="str">
+        <v>Fail</v>
+      </c>
+      <c r="H80" t="str">
+        <v>Search_VoiceSearchFake.png</v>
+      </c>
+      <c r="I80" t="str">
+        <v>Voice search is simulated - always returns "plumber" after timeout</v>
+      </c>
+      <c r="J80" t="str">
+        <v>Implement real Web Speech API SpeechRecognition integration</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>TC080</v>
+      </c>
+      <c r="B81" t="str">
+        <v>Auth</v>
+      </c>
+      <c r="C81" t="str">
+        <v>Admin Login</v>
+      </c>
+      <c r="D81" t="str">
+        <v>Admin org code validated server-side</v>
+      </c>
+      <c r="E81" t="str">
+        <v>Organization code verified against database</v>
+      </c>
+      <c r="F81" t="str">
+        <v>Organization code stored in sessionStorage but never validated server-side. Any code accepted.</v>
+      </c>
+      <c r="G81" t="str">
+        <v>Fail</v>
+      </c>
+      <c r="H81" t="str">
+        <v>AdminLogin_OrgCodeNotValidated.png</v>
+      </c>
+      <c r="I81" t="str">
+        <v>Organization code provides no real security - never verified</v>
+      </c>
+      <c r="J81" t="str">
+        <v>Add server-side org code validation against admin organizations table</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>TC081</v>
+      </c>
+      <c r="B82" t="str">
+        <v>Middleware</v>
+      </c>
+      <c r="C82" t="str">
+        <v>Rate Limiting</v>
+      </c>
+      <c r="D82" t="str">
+        <v>Rate limiting persists across server restarts</v>
+      </c>
+      <c r="E82" t="str">
+        <v>Rate limit state stored in Redis or persistent store</v>
+      </c>
+      <c r="F82" t="str">
+        <v>Rate limiting uses in-memory Map (globalThis). Resets on server restart. Ineffective in multi-instance deploy.</v>
+      </c>
+      <c r="G82" t="str">
+        <v>Fail</v>
+      </c>
+      <c r="H82" t="str">
+        <v>Middleware_InMemoryRateLimit.png</v>
+      </c>
+      <c r="I82" t="str">
+        <v>In-memory rate limiting resets on restart and doesnt work across instances</v>
+      </c>
+      <c r="J82" t="str">
+        <v>Use Redis or similar distributed store for rate limiting</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J64"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J82"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add critical broken link findings: /auth/login routes do not exist
New findings from navigation audit:
- Menu sign-out button routes to /auth/login (page does NOT exist) - should be /login
- Admin login back-link routes to /auth/login (page does NOT exist) - should be /login

Updated totals: 83 test cases, 22 broken link checks, 56.6% pass rate

https://claude.ai/code/session_01RGfJPwNgYTYKFEZvETDMzN
</commit_message>
<xml_diff>
--- a/QA_Reports/QA_Report.xlsx
+++ b/QA_Reports/QA_Report.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J82"/>
+  <dimension ref="A1:J84"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -3036,16 +3036,80 @@
         <v>Use Redis or similar distributed store for rate limiting</v>
       </c>
     </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>TC082</v>
+      </c>
+      <c r="B83" t="str">
+        <v>Navigation</v>
+      </c>
+      <c r="C83" t="str">
+        <v>Menu</v>
+      </c>
+      <c r="D83" t="str">
+        <v>Sign out redirects to login page</v>
+      </c>
+      <c r="E83" t="str">
+        <v>User redirected to /login after sign out</v>
+      </c>
+      <c r="F83" t="str">
+        <v>Sign out button routes to /auth/login which does NOT exist as a page. Correct path is /login.</v>
+      </c>
+      <c r="G83" t="str">
+        <v>Fail</v>
+      </c>
+      <c r="H83" t="str">
+        <v>Menu_SignOut_BrokenLink.png</v>
+      </c>
+      <c r="I83" t="str">
+        <v>Wrong path /auth/login used instead of /login in menu/page.tsx line 203</v>
+      </c>
+      <c r="J83" t="str">
+        <v>Change router.push path from /auth/login to /login</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>TC083</v>
+      </c>
+      <c r="B84" t="str">
+        <v>Navigation</v>
+      </c>
+      <c r="C84" t="str">
+        <v>Admin Login</v>
+      </c>
+      <c r="D84" t="str">
+        <v>Back to login link works</v>
+      </c>
+      <c r="E84" t="str">
+        <v>Link navigates to /login page</v>
+      </c>
+      <c r="F84" t="str">
+        <v>Routes to /auth/login which does NOT exist. admin-login/page.tsx line 49</v>
+      </c>
+      <c r="G84" t="str">
+        <v>Fail</v>
+      </c>
+      <c r="H84" t="str">
+        <v>AdminLogin_BackLink_Broken.png</v>
+      </c>
+      <c r="I84" t="str">
+        <v>Wrong path /auth/login instead of /login</v>
+      </c>
+      <c r="J84" t="str">
+        <v>Change href from /auth/login to /login</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J82"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J84"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G23"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="25.83203125" customWidth="1"/>
@@ -3081,108 +3145,108 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>TopNav</v>
+        <v>Menu</v>
       </c>
       <c r="B2" t="str">
-        <v>Notification Bell</v>
+        <v>Sign Out Button</v>
       </c>
       <c r="C2" t="str">
-        <v>/notifications page opens</v>
+        <v>Redirects to /login</v>
       </c>
       <c r="D2" t="str">
-        <v>Navigates to /notifications correctly, BUT active state check uses /notification (missing s) - never highlights as active</v>
+        <v>Routes to /auth/login which does NOT exist. Correct path is /login. menu/page.tsx line 203</v>
       </c>
       <c r="E2" t="str">
         <v>Fail</v>
       </c>
       <c r="F2" t="str">
-        <v>TopNav_NotificationActive_Bug.png</v>
+        <v>Menu_SignOut_BrokenLink.png</v>
       </c>
       <c r="G2" t="str">
-        <v>Fix pathname check from /notification to /notifications in TopNav.tsx line 81</v>
+        <v>Change /auth/login to /login in menu/page.tsx line 203</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>TopNav</v>
+        <v>Admin Login</v>
       </c>
       <c r="B3" t="str">
-        <v>Netyard Tab</v>
+        <v>Back to Login link</v>
       </c>
       <c r="C3" t="str">
-        <v>/netyard or /community page</v>
+        <v>Redirects to /login</v>
       </c>
       <c r="D3" t="str">
-        <v>Links to /netyard which exists, but /community is a separate page - potential user confusion about which is the main community page</v>
+        <v>Routes to /auth/login which does NOT exist. admin-login/page.tsx line 49</v>
       </c>
       <c r="E3" t="str">
-        <v>Warning</v>
+        <v>Fail</v>
       </c>
       <c r="F3" t="str">
-        <v>TopNav_Netyard_Community_Confusion.png</v>
+        <v>AdminLogin_BackLink_Broken.png</v>
       </c>
       <c r="G3" t="str">
-        <v>Consolidate /netyard and /community or clarify naming</v>
+        <v>Change /auth/login to /login in admin-login/page.tsx line 49</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ChatBot</v>
+        <v>TopNav</v>
       </c>
       <c r="B4" t="str">
-        <v>Quick Action - Find Workers</v>
+        <v>Notification Bell</v>
       </c>
       <c r="C4" t="str">
-        <v>/jobplace/providers opens</v>
+        <v>/notifications page opens</v>
       </c>
       <c r="D4" t="str">
-        <v>Navigation link in chatbot response directs to /jobplace/providers correctly</v>
+        <v>Navigates to /notifications correctly, BUT active state check uses /notification (missing s) - never highlights as active</v>
       </c>
       <c r="E4" t="str">
-        <v>Pass</v>
+        <v>Fail</v>
       </c>
       <c r="F4" t="str">
-        <v>N/A</v>
+        <v>TopNav_NotificationActive_Bug.png</v>
       </c>
       <c r="G4" t="str">
-        <v/>
+        <v>Fix pathname check from /notification to /notifications in TopNav.tsx line 81</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ChatBot</v>
+        <v>TopNav</v>
       </c>
       <c r="B5" t="str">
-        <v>Quick Action - Map</v>
+        <v>Netyard Tab</v>
       </c>
       <c r="C5" t="str">
-        <v>/jobplace/map opens</v>
+        <v>/netyard or /community page</v>
       </c>
       <c r="D5" t="str">
-        <v>Navigation link works correctly</v>
+        <v>Links to /netyard which exists, but /community is a separate page - potential user confusion about which is the main community page</v>
       </c>
       <c r="E5" t="str">
-        <v>Pass</v>
+        <v>Warning</v>
       </c>
       <c r="F5" t="str">
-        <v>N/A</v>
+        <v>TopNav_Netyard_Community_Confusion.png</v>
       </c>
       <c r="G5" t="str">
-        <v/>
+        <v>Consolidate /netyard and /community or clarify naming</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Home Feed</v>
+        <v>ChatBot</v>
       </c>
       <c r="B6" t="str">
-        <v>Create Post - Job Link</v>
+        <v>Quick Action - Find Workers</v>
       </c>
       <c r="C6" t="str">
-        <v>/jobplace/create opens</v>
+        <v>/jobplace/providers opens</v>
       </c>
       <c r="D6" t="str">
-        <v>Link to /jobplace/create works, page exists</v>
+        <v>Navigation link in chatbot response directs to /jobplace/providers correctly</v>
       </c>
       <c r="E6" t="str">
         <v>Pass</v>
@@ -3196,16 +3260,16 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Menu</v>
+        <v>ChatBot</v>
       </c>
       <c r="B7" t="str">
-        <v>Search Button</v>
+        <v>Quick Action - Map</v>
       </c>
       <c r="C7" t="str">
-        <v>/search page opens</v>
+        <v>/jobplace/map opens</v>
       </c>
       <c r="D7" t="str">
-        <v>router.push(/search) works correctly</v>
+        <v>Navigation link works correctly</v>
       </c>
       <c r="E7" t="str">
         <v>Pass</v>
@@ -3219,16 +3283,16 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Menu</v>
+        <v>Home Feed</v>
       </c>
       <c r="B8" t="str">
-        <v>Various Menu Items</v>
+        <v>Create Post - Job Link</v>
       </c>
       <c r="C8" t="str">
-        <v>All menu items navigate to correct pages</v>
+        <v>/jobplace/create opens</v>
       </c>
       <c r="D8" t="str">
-        <v>Menu items link to various pages. All verified to exist as page routes</v>
+        <v>Link to /jobplace/create works, page exists</v>
       </c>
       <c r="E8" t="str">
         <v>Pass</v>
@@ -3242,16 +3306,16 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Profile</v>
+        <v>Menu</v>
       </c>
       <c r="B9" t="str">
-        <v>Edit Profile</v>
+        <v>Search Button</v>
       </c>
       <c r="C9" t="str">
-        <v>/profile/edit opens</v>
+        <v>/search page opens</v>
       </c>
       <c r="D9" t="str">
-        <v>router.push(/profile/edit) works correctly</v>
+        <v>router.push(/search) works correctly</v>
       </c>
       <c r="E9" t="str">
         <v>Pass</v>
@@ -3265,16 +3329,16 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Settings</v>
+        <v>Menu</v>
       </c>
       <c r="B10" t="str">
-        <v>Account Settings</v>
+        <v>Various Menu Items</v>
       </c>
       <c r="C10" t="str">
-        <v>/settings/account opens</v>
+        <v>All menu items navigate to correct pages</v>
       </c>
       <c r="D10" t="str">
-        <v>Navigation works correctly</v>
+        <v>Menu items link to various pages. All verified to exist as page routes</v>
       </c>
       <c r="E10" t="str">
         <v>Pass</v>
@@ -3288,16 +3352,16 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Settings</v>
+        <v>Profile</v>
       </c>
       <c r="B11" t="str">
-        <v>Activity Log</v>
+        <v>Edit Profile</v>
       </c>
       <c r="C11" t="str">
-        <v>/settings/activity opens</v>
+        <v>/profile/edit opens</v>
       </c>
       <c r="D11" t="str">
-        <v>router.push(/settings/activity) works correctly</v>
+        <v>router.push(/profile/edit) works correctly</v>
       </c>
       <c r="E11" t="str">
         <v>Pass</v>
@@ -3314,13 +3378,13 @@
         <v>Settings</v>
       </c>
       <c r="B12" t="str">
-        <v>Privacy Policy</v>
+        <v>Account Settings</v>
       </c>
       <c r="C12" t="str">
-        <v>/privacy page opens</v>
+        <v>/settings/account opens</v>
       </c>
       <c r="D12" t="str">
-        <v>Navigation to /privacy works, page exists</v>
+        <v>Navigation works correctly</v>
       </c>
       <c r="E12" t="str">
         <v>Pass</v>
@@ -3337,36 +3401,36 @@
         <v>Settings</v>
       </c>
       <c r="B13" t="str">
-        <v>Terms of Service</v>
+        <v>Activity Log</v>
       </c>
       <c r="C13" t="str">
-        <v>/terms page opens</v>
+        <v>/settings/activity opens</v>
       </c>
       <c r="D13" t="str">
-        <v>No /terms page found in the application routes</v>
+        <v>router.push(/settings/activity) works correctly</v>
       </c>
       <c r="E13" t="str">
-        <v>Fail</v>
+        <v>Pass</v>
       </c>
       <c r="F13" t="str">
-        <v>Settings_TermsLink_Broken.png</v>
+        <v>N/A</v>
       </c>
       <c r="G13" t="str">
-        <v>Create /terms page or remove the link</v>
+        <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Auth/Login</v>
+        <v>Settings</v>
       </c>
       <c r="B14" t="str">
-        <v>Login Redirect</v>
+        <v>Privacy Policy</v>
       </c>
       <c r="C14" t="str">
-        <v>/home after successful login</v>
+        <v>/privacy page opens</v>
       </c>
       <c r="D14" t="str">
-        <v>Redirect to /home after auth works correctly</v>
+        <v>Navigation to /privacy works, page exists</v>
       </c>
       <c r="E14" t="str">
         <v>Pass</v>
@@ -3380,39 +3444,39 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Middleware</v>
+        <v>Settings</v>
       </c>
       <c r="B15" t="str">
-        <v>Auth Redirect</v>
+        <v>Terms of Service</v>
       </c>
       <c r="C15" t="str">
-        <v>/login for unauthenticated users</v>
+        <v>/terms page opens</v>
       </c>
       <c r="D15" t="str">
-        <v>Protected routes redirect to /login correctly</v>
+        <v>No /terms page found in the application routes</v>
       </c>
       <c r="E15" t="str">
-        <v>Pass</v>
+        <v>Fail</v>
       </c>
       <c r="F15" t="str">
-        <v>N/A</v>
+        <v>Settings_TermsLink_Broken.png</v>
       </c>
       <c r="G15" t="str">
-        <v/>
+        <v>Create /terms page or remove the link</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Home Feed</v>
+        <v>Auth/Login</v>
       </c>
       <c r="B16" t="str">
-        <v>Community Groups Section</v>
+        <v>Login Redirect</v>
       </c>
       <c r="C16" t="str">
-        <v>/community page opens</v>
+        <v>/home after successful login</v>
       </c>
       <c r="D16" t="str">
-        <v>Link to /community works correctly</v>
+        <v>Redirect to /home after auth works correctly</v>
       </c>
       <c r="E16" t="str">
         <v>Pass</v>
@@ -3426,16 +3490,16 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Various Pages</v>
+        <v>Middleware</v>
       </c>
       <c r="B17" t="str">
-        <v>router.back()</v>
+        <v>Auth Redirect</v>
       </c>
       <c r="C17" t="str">
-        <v>Previous page in browser history</v>
+        <v>/login for unauthenticated users</v>
       </c>
       <c r="D17" t="str">
-        <v>Multiple pages use router.back() - works as expected via Next.js router</v>
+        <v>Protected routes redirect to /login correctly</v>
       </c>
       <c r="E17" t="str">
         <v>Pass</v>
@@ -3449,39 +3513,39 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>JobPlace</v>
+        <v>Home Feed</v>
       </c>
       <c r="B18" t="str">
-        <v>Job Detail Link</v>
+        <v>Community Groups Section</v>
       </c>
       <c r="C18" t="str">
-        <v>/jobplace/job/[id] opens</v>
+        <v>/community page opens</v>
       </c>
       <c r="D18" t="str">
-        <v>Hardcoded link to /jobplace/job/1 found in code - should use dynamic ID</v>
+        <v>Link to /community works correctly</v>
       </c>
       <c r="E18" t="str">
-        <v>Warning</v>
+        <v>Pass</v>
       </c>
       <c r="F18" t="str">
-        <v>JobPlace_HardcodedJobLink.png</v>
+        <v>N/A</v>
       </c>
       <c r="G18" t="str">
-        <v>Use dynamic job ID instead of hardcoded /jobplace/job/1</v>
+        <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>BottomNav</v>
+        <v>Various Pages</v>
       </c>
       <c r="B19" t="str">
-        <v>Reels Tab</v>
+        <v>router.back()</v>
       </c>
       <c r="C19" t="str">
-        <v>/reels page opens</v>
+        <v>Previous page in browser history</v>
       </c>
       <c r="D19" t="str">
-        <v>Navigation to /reels works correctly</v>
+        <v>Multiple pages use router.back() - works as expected via Next.js router</v>
       </c>
       <c r="E19" t="str">
         <v>Pass</v>
@@ -3495,53 +3559,99 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>BottomNav</v>
+        <v>JobPlace</v>
       </c>
       <c r="B20" t="str">
-        <v>Community Tab</v>
+        <v>Job Detail Link</v>
       </c>
       <c r="C20" t="str">
-        <v>/community page opens</v>
+        <v>/jobplace/job/[id] opens</v>
       </c>
       <c r="D20" t="str">
-        <v>BottomNav links to /community, but TopNav links to /netyard for the same concept</v>
+        <v>Hardcoded link to /jobplace/job/1 found in code - should use dynamic ID</v>
       </c>
       <c r="E20" t="str">
         <v>Warning</v>
       </c>
       <c r="F20" t="str">
-        <v>Nav_CommunityPath_Inconsistent.png</v>
+        <v>JobPlace_HardcodedJobLink.png</v>
       </c>
       <c r="G20" t="str">
-        <v>Both navs should link to same community path</v>
+        <v>Use dynamic job ID instead of hardcoded /jobplace/job/1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
+        <v>BottomNav</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Reels Tab</v>
+      </c>
+      <c r="C21" t="str">
+        <v>/reels page opens</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Navigation to /reels works correctly</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="F21" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="G21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>BottomNav</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Community Tab</v>
+      </c>
+      <c r="C22" t="str">
+        <v>/community page opens</v>
+      </c>
+      <c r="D22" t="str">
+        <v>BottomNav links to /community, but TopNav links to /netyard for the same concept</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Warning</v>
+      </c>
+      <c r="F22" t="str">
+        <v>Nav_CommunityPath_Inconsistent.png</v>
+      </c>
+      <c r="G22" t="str">
+        <v>Both navs should link to same community path</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
         <v>Home Feed</v>
       </c>
-      <c r="B21" t="str">
+      <c r="B23" t="str">
         <v>Inbox Link</v>
       </c>
-      <c r="C21" t="str">
+      <c r="C23" t="str">
         <v>/inbox page opens</v>
       </c>
-      <c r="D21" t="str">
+      <c r="D23" t="str">
         <v>Both /inbox and /messages exist as separate pages for messaging - inconsistent entry points</v>
       </c>
-      <c r="E21" t="str">
+      <c r="E23" t="str">
         <v>Warning</v>
       </c>
-      <c r="F21" t="str">
+      <c r="F23" t="str">
         <v>Messages_DualEntryPoints.png</v>
       </c>
-      <c r="G21" t="str">
+      <c r="G23" t="str">
         <v>Consolidate /inbox and /messages into single messaging entry point</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G23"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>